<commit_message>
Rerun week ending 24-Jul-26 against primary sources
Network access to the wires and trade press was opened, so every row was
re-verified against the originating release rather than search summaries:

- Add Neo ($100m, a16z/Bessemer, out of stealth 20-Jul) - missed on the
  first pass, confirmed via GlobeNewswire and the FinTech Global weekly
- Correct Genki/Wave Claims to 19-Jul-26 per the PRWeb Cologne dateline
  (21-Jul was the trade-press pickup date, not the announcement)
- Correct Natural to 20-Jul-26 per the PR Newswire release
- Add EV/Revenue 5.8x for Genius AI ($1.15bn valuation on a ~$200m
  revenue run-rate)
- Note FinWise/Tallied structure as an acquisition-and-assumption of the
  platform and related assets, per the Form 8-K

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134qWJfn5kVUs6bAvN1m6Pd
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0&quot;x&quot;"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -79,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -89,6 +91,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -594,7 +599,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-26</t>
+          <t>19-Jul-26</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -712,7 +717,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Credit card issuing and processing platform spanning application, issuing, processing and servicing; FinWise bought the platform and related assets to own its card stack end-to-end</t>
+          <t>Credit card issuing and processing platform spanning application, issuing, processing and servicing; structured as an acquisition-and-assumption of the platform and related assets rather than a share purchase</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -762,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -986,21 +991,21 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-26</t>
+          <t>20-Jul-26</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Empirical Security</t>
+          <t>Neo</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Brightmind Partners</t>
+          <t>Andreessen Horowitz, Bessemer Venture Partners</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1019,7 +1024,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>AI exposure-management platform that predicts which vulnerabilities will actually be exploited and prioritises remediation</t>
+          <t>Real-time control layer that inventories and governs AI agents, agentic applications and MCP servers across an enterprise software estate; launched out of stealth</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1047,24 +1052,26 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>22-Jul-26</t>
+          <t>21-Jul-26</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Glow</t>
+          <t>Empirical Security</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sequoia Capital, Cyberstarts</t>
+          <t>Brightmind Partners</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>180</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1200</v>
+        <v>25</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -1078,7 +1085,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>AI-native, prevention-first endpoint security platform; launched out of stealth</t>
+          <t>AI exposure-management platform that predicts which vulnerabilities will actually be exploited and prioritises remediation</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -1106,26 +1113,24 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>23-Jul-26</t>
+          <t>22-Jul-26</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Glow</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Cheyenne Ventures, AVP</t>
+          <t>Sequoia Capital, Cyberstarts</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>180</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1200</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1144,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
+          <t>AI-native, prevention-first endpoint security platform; launched out of stealth</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1157,31 +1162,31 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>20-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Ant International</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Ant Group, Alibaba Group</t>
+          <t>Cheyenne Ventures, AVP</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1200</v>
+        <v>25</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -1200,7 +1205,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
+          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1223,29 +1228,31 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-26</t>
+          <t>20-Jul-26</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Genius AI (GlossGenius)</t>
+          <t>Ant International</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Lux Capital</t>
+          <t>Ant Group, Alibaba Group</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>1150</v>
+        <v>1200</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1259,7 +1266,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses, facilitating ~$7bn of annual sales across 125,000 merchants</t>
+          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1287,7 +1294,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-26</t>
+          <t>20-Jul-26</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1329,8 +1336,65 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>24-Jul-26</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>21-Jul-26</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Genius AI (GlossGenius)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Lux Capital</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1150</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses, facilitating ~$7bn of annual sales across 125,000 merchants</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M9"/>
+  <autoFilter ref="A1:M10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -1340,6 +1404,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Corgi Series B extension to week ending 24-Jul-26
Included at the user's direction despite an undisclosed round size, so
the row carries valuation ($4bn) with Amount and Lead Investor(s) as "-"
and the structure noted in the description.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134qWJfn5kVUs6bAvN1m6Pd
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -767,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1223,36 +1223,36 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>20-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Ant International</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Ant Group, Alibaba Group</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>4000</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
+          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover; further Series B extension, size and investors undisclosed</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1299,16 +1299,16 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Ant International</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Forerunner Ventures</t>
+          <t>Ant Group, Alibaba Group</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
+          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1355,46 +1355,107 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>20-Jul-26</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Forerunner Ventures</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>24-Jul-26</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>21-Jul-26</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Genius AI (GlossGenius)</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Lux Capital</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I11" s="2" t="n">
         <v>1150</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>5.8</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Booking, payments and business-management platform for in-person beauty and wellness businesses, facilitating ~$7bn of annual sales across 125,000 merchants</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M10"/>
+  <autoFilter ref="A1:M11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -1405,6 +1466,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add three deals surfaced from PitchBook Daily Pitch, week ending 24-Jul-26
None of these appeared in the fintech trade press sweep:

- AEGIS Hedging Solutions / Private Equity at Goldman Sachs Alternatives
  (22-Jul, PE Buyout) - commodity price-risk technology, terms undisclosed
- AegisAI $36m Series A led by Battery Ventures (23-Jul) - anti-phishing,
  consistent with the DB's existing enterprise-security precedent
- Street Group / Hg (22-Jul) - booked as a raise, not M&A: founders remain
  majority holders, so it is a minority growth investment. Valuation
  converted from the GBP200m+ headline at 1.3375 on the announcement date

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134qWJfn5kVUs6bAvN1m6Pd
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -584,32 +584,32 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>PE Buyout</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>19-Jul-26</t>
+          <t>22-Jul-26</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Wave Claims (Claim OS)</t>
+          <t>AEGIS Hedging Solutions</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Genki</t>
+          <t>Private Equity at Goldman Sachs Alternatives</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>AI claims-automation platform (Claim OS) that reads medical invoices, structures claims data, assigns ICD diagnosis codes and flags potential fraud for health insurers</t>
+          <t>Commodity price-risk platform pairing hedging technology and market intelligence for ~700 producers, consumers, capital providers and financial counterparties across North America</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -672,90 +672,179 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>19-Jul-26</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Wave Claims (Claim OS)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Genki</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>AI claims-automation platform (Claim OS) that reads medical invoices, structures claims data, assigns ICD diagnosis codes and flags potential fraud for health insurers</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>24-Jul-26</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Strategic M&amp;A</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>20-Jul-26</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Tallied Technologies (platform)</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>FinWise Bancorp</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Credit card issuing and processing platform spanning application, issuing, processing and servicing; structured as an acquisition-and-assumption of the platform and related assets rather than a share purchase</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Tallied Technologies, Inc.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R3"/>
+  <autoFilter ref="A1:R4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -767,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1177,16 +1266,16 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>AegisAI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Cheyenne Ventures, AVP</t>
+          <t>Battery Ventures</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -1205,7 +1294,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
+          <t>AI agents that detect and block AI-generated spear-phishing and business email compromise</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1223,7 +1312,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1238,21 +1327,21 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Corgi</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>4000</v>
+          <t>Cheyenne Ventures, AVP</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1266,7 +1355,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover; further Series B extension, size and investors undisclosed</t>
+          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1284,36 +1373,36 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>20-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Ant International</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Ant Group, Alibaba Group</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>4000</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -1327,7 +1416,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
+          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover; further Series B extension, size and investors undisclosed</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1350,7 +1439,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1360,16 +1449,16 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Ant International</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Forerunner Ventures</t>
+          <t>Ant Group, Alibaba Group</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>30</v>
+        <v>1200</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1388,7 +1477,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
+          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -1416,46 +1505,168 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>20-Jul-26</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Forerunner Ventures</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24-Jul-26</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>21-Jul-26</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Genius AI (GlossGenius)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Lux Capital</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I12" s="2" t="n">
         <v>1150</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>5.8</v>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Booking, payments and business-management platform for in-person beauty and wellness businesses, facilitating ~$7bn of annual sales across 125,000 merchants</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>24-Jul-26</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>22-Jul-26</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Street Group</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Hg</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>268</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Vertical software and AI operating system for UK estate and letting agents; minority growth investment at a £200m+ valuation (converted at 1.3375 on 22-Jul), founders retain control</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M11"/>
+  <autoFilter ref="A1:M13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -1467,6 +1678,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Trim scale trivia and round-status padding from descriptions
Two patterns get deleted by hand every week, so encode them as rules
rather than fixing them per-run:

- Rule 3 now covers volume metrics (TPV, GMV, sales facilitated,
  merchant/user counts, AUM), not just client counts and geography
- New rule 4 bans round/deal status entirely ("launched out of stealth",
  "size and investors undisclosed", "terms undisclosed") - the Amount,
  Valuation and EV columns already carry that, and a dash is itself the
  disclosure
- Rule 7 narrows the structure-nuance exception to cases where the note
  explains why a column reads the way it does

All 15 rows for the week ending 24-Jul-26 rewritten to match; every
description now sits in the 5-21 word band.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134qWJfn5kVUs6bAvN1m6Pd
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
@@ -629,7 +629,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Commodity price-risk platform pairing hedging technology and market intelligence for ~700 producers, consumers, capital providers and financial counterparties across North America</t>
+          <t>Commodity price-risk platform pairing hedging technology with market intelligence</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>AI claims-automation platform (Claim OS) that reads medical invoices, structures claims data, assigns ICD diagnosis codes and flags potential fraud for health insurers</t>
+          <t>AI claims-automation platform (Claim OS) that reads medical invoices, structures claims data, assigns ICD codes and flags potential fraud</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Credit card issuing and processing platform spanning application, issuing, processing and servicing; structured as an acquisition-and-assumption of the platform and related assets rather than a share purchase</t>
+          <t>Credit card issuing and processing platform spanning application, issuing, processing and servicing; bought as a platform-and-assets purchase, not a share deal</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Interest-free BNPL and consumer credit platform with 10m+ accounts and 40,000 merchants in Venezuela; $80m equity across combined Series A and B ($100m headline includes $20m debt)</t>
+          <t>Interest-free BNPL and consumer credit platform in Venezuela; $80m equity of the $100m headline</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Real-time control layer that inventories and governs AI agents, agentic applications and MCP servers across an enterprise software estate; launched out of stealth</t>
+          <t>Real-time control layer that inventories and governs AI agents, agentic applications and MCP servers across an enterprise software estate</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>AI-native, prevention-first endpoint security platform; launched out of stealth</t>
+          <t>AI-native, prevention-first endpoint security platform</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover; further Series B extension, size and investors undisclosed</t>
+          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr, connecting 150m+ merchants to 2bn digital accounts</t>
+          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses, facilitating ~$7bn of annual sales across 125,000 merchants</t>
+          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Vertical software and AI operating system for UK estate and letting agents; minority growth investment at a £200m+ valuation (converted at 1.3375 on 22-Jul), founders retain control</t>
+          <t>Vertical software and AI operating system for UK estate and letting agents; minority investment, founders retain control</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Calibrate CyberTech scope; drop Glow, Neo and Empirical Security
Keeping AegisAI and Abstract implies the boundary is not deal size and
not a strict financial nexus (Abstract has none). The rule that fits both
keeps: a security deal qualifies on a financial-crime/fraud nexus OR on
being genuinely a data/analytics platform, which is what the sector label
says. Pure security-operations tooling - endpoint, vulnerability and
exposure management, agent control planes, defense - is out.

Applied to the week ending 24-Jul-26: Glow ($180m endpoint), Neo ($100m
agent control layer) and Empirical Security ($25m exposure prediction)
come out. Raises go 12 -> 9 and disclosed volume $1.90bn -> $1.60bn.

Recorded as rule 6 in SKILL.md, with the note that roundup CyberTech
coverage is not to be inherited wholesale - that is how the sector drifted.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134qWJfn5kVUs6bAvN1m6Pd
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-24.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -856,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1080,21 +1080,21 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>20-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Neo</t>
+          <t>AegisAI</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Andreessen Horowitz, Bessemer Venture Partners</t>
+          <t>Battery Ventures</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Real-time control layer that inventories and governs AI agents, agentic applications and MCP servers across an enterprise software estate</t>
+          <t>AI agents that detect and block AI-generated spear-phishing and business email compromise</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1141,17 +1141,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Empirical Security</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Brightmind Partners</t>
+          <t>Cheyenne Ventures, AVP</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>AI exposure-management platform that predicts which vulnerabilities will actually be exploited and prioritises remediation</t>
+          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1202,24 +1202,26 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>22-Jul-26</t>
+          <t>23-Jul-26</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Glow</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Sequoia Capital, Cyberstarts</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>180</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1200</v>
+        <v>4000</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -1233,7 +1235,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>AI-native, prevention-first endpoint security platform</t>
+          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1251,31 +1253,31 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>23-Jul-26</t>
+          <t>20-Jul-26</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AegisAI</t>
+          <t>Ant International</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Battery Ventures</t>
+          <t>Ant Group, Alibaba Group</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>36</v>
+        <v>1200</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -1294,7 +1296,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>AI agents that detect and block AI-generated spear-phishing and business email compromise</t>
+          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1312,7 +1314,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1322,21 +1324,21 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>23-Jul-26</t>
+          <t>20-Jul-26</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Natural</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Cheyenne Ventures, AVP</t>
+          <t>Forerunner Ventures</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1355,7 +1357,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Composable, streaming-first security operations platform built to displace monolithic SIEM</t>
+          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1373,7 +1375,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1383,31 +1385,27 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>23-Jul-26</t>
+          <t>21-Jul-26</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Corgi</t>
+          <t>Genius AI (GlossGenius)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Lux Capital</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>44</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1150</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>5.8</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1416,7 +1414,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Full-stack AI insurance platform spanning underwriting, claims and embedded commercial cover</t>
+          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1434,36 +1432,36 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Real Estate &amp; Mortgage Tech</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>20-Jul-26</t>
+          <t>22-Jul-26</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Ant International</t>
+          <t>Street Group</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Ant Group, Alibaba Group</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Hg</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>268</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -1477,196 +1475,17 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments and digital financial services group operating Alipay+, Antom, WorldFirst and Bettr</t>
+          <t>Vertical software and AI operating system for UK estate and letting agents; minority investment, founders retain control</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>24-Jul-26</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>20-Jul-26</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Natural</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Forerunner Ventures</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Payments infrastructure letting AI agents hold wallets, accept payments, pay invoices and settle transactions autonomously</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>24-Jul-26</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>21-Jul-26</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Genius AI (GlossGenius)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Lux Capital</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>1150</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Booking, payments and business-management platform for in-person beauty and wellness businesses</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>24-Jul-26</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>22-Jul-26</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Street Group</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Hg</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>268</v>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Vertical software and AI operating system for UK estate and letting agents; minority investment, founders retain control</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M13"/>
+  <autoFilter ref="A1:M10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -1677,9 +1496,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>